<commit_message>
Alle coördinaten systematisch vervangen met exacte locaties
</commit_message>
<xml_diff>
--- a/zorginstellingen data.xlsx
+++ b/zorginstellingen data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10601"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mhakeizer/Downloads/GGZjeugdAmsterdam/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BDF6D0F8-1719-D544-BD68-FF5476E5512F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCA4C0DB-7508-7F48-A3CA-F15BD8CC2C39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{BF594656-5C97-1D46-8141-67E1D0E71DE6}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16120" xr2:uid="{BF594656-5C97-1D46-8141-67E1D0E71DE6}"/>
   </bookViews>
   <sheets>
     <sheet name="zorginstellingen" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="283">
   <si>
     <t>Naam</t>
   </si>
@@ -869,6 +869,9 @@
   </si>
   <si>
     <t>020 – 49 41 296</t>
+  </si>
+  <si>
+    <t>Naam op de kaart</t>
   </si>
 </sst>
 </file>
@@ -1758,8 +1761,9 @@
     <col min="4" max="4" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="74.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="48" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="54.1640625" customWidth="1"/>
     <col min="8" max="8" width="44" customWidth="1"/>
+    <col min="9" max="9" width="98.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
@@ -1790,6 +1794,9 @@
       <c r="I1" t="s">
         <v>131</v>
       </c>
+      <c r="J1" t="s">
+        <v>282</v>
+      </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -1946,6 +1953,9 @@
       </c>
       <c r="I6" t="s">
         <v>92</v>
+      </c>
+      <c r="J6" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">

</xml_diff>